<commit_message>
fix(quiz): audit and update 395 quiz answers and explanations across all 15 days
</commit_message>
<xml_diff>
--- a/TONG_HOP_QUIZ_15_NGAY_EXCEL/01_CHUAN_IMPORT_QUIZIZZ_QUIZ_COM_904_CAU/Day_01_Giới thiệu _ Foundation LLM/Day_01_FULL_TOAN_BO_101_CAU.xlsx
+++ b/TONG_HOP_QUIZ_15_NGAY_EXCEL/01_CHUAN_IMPORT_QUIZIZZ_QUIZ_COM_904_CAU/Day_01_Giới thiệu _ Foundation LLM/Day_01_FULL_TOAN_BO_101_CAU.xlsx
@@ -796,7 +796,7 @@
       </c>
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>60</v>
@@ -804,7 +804,7 @@
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Xem hệ thống chỉ tạo một đầu ra hay còn quan sát và hành động qua nhiều bước để đạt mục tiêu.</t>
+          <t>Hệ thống nhận mục tiêu, tự kiểm tra lịch của 4 người, đề xuất giờ, gửi lời mời qua công cụ và xác nhận trạng thái là hệ thống có hành vi tác nhân (agentic) vì nó tự lập kế hoạch và hành động qua nhiều bước để đạt mục tiêu.</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>3,4</t>
+          <t>1,3</t>
         </is>
       </c>
       <c r="I7" s="4" t="n">
@@ -859,7 +859,7 @@
       <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Đừng gọi một hệ thống là agent chỉ vì nó có thể sinh nội dung. Tìm các trường hợp tạo nội dung mới rồi kết thúc sau một lượt xử lý.</t>
+          <t>Mô hình viết đoạn mô tả từ yêu cầu rồi kết thúc (a) và mô hình tạo ảnh từ mô tả rồi kết thúc (c) là các hệ thống sinh nội dung (generative) nhưng chỉ chạy một lượt và không có vòng lặp kế hoạch, công cụ hay trạng thái của một agent.</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>60</v>
@@ -907,7 +907,7 @@
       <c r="J8" s="3" t="n"/>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: So sánh việc viết quy tắc thủ công với việc để mô hình học biểu diễn từ dữ liệu.</t>
+          <t>Mô hình tạo sinh quy mô lớn thành công nhờ khả năng học biểu diễn từ lượng dữ liệu khổng lồ bằng năng lực tính toán và kiến trúc Transformer, chứ không phải do mở rộng các bộ quy tắc thủ công của con người.</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>3,5</t>
+          <t>1,2,3</t>
         </is>
       </c>
       <c r="I10" s="4" t="n">
@@ -1020,7 +1020,7 @@
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tách chức năng do ứng dụng tổ chức quanh mô hình khỏi cơ chế bên trong chính mô hình đó.</t>
+          <t>Khi thay thế foundation model, lớp ứng dụng/sản phẩm cần tự vận hành gồm: Xác thực và hạn ngạch người dùng (a), Giao diện trò chuyện (b), và Quy tắc kiểm duyệt nội dung của ứng dụng (c). Cơ chế attention và trọng số thuộc về chính mô hình nền tảng.</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11" s="4" t="n">
         <v>60</v>
@@ -1068,7 +1068,7 @@
       <c r="J11" s="3" t="n"/>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tìm đặc điểm cho phép hệ thống tiếp tục hành động sau phản hồi đầu tiên.</t>
+          <t>Hệ thống A chỉ gọi LLM một lượt để viết email nên là ứng dụng gọi LLM đơn thuần; Hệ thống B có mục tiêu, kế hoạch, công cụ (CRM, lịch) và trạng thái nên là một agent đầy đủ.</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>o1 → o2 → o3 → o4 → o5</t>
+          <t>o2 → o3 → o1 → o4 → o5</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1226,7 +1226,7 @@
       <c r="J14" s="3" t="n"/>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Không cập nhật trạng thái đặt vé trước khi công cụ xác nhận đổi vé thành công.</t>
+          <t>Vòng xử lý hợp lý bắt đầu từ lập kế hoạch gọi công cụ đổi vé (o2) -&gt; thực thi gọi công cụ ticket.change (o3) -&gt; nhận kết quả đổi vé thành công X9 (o1) -&gt; cập nhật trạng thái đặt vé thành X9 (o4) -&gt; thông báo kết quả rồi dừng (o5).</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I16" s="4" t="n">
         <v>60</v>
@@ -1324,7 +1324,7 @@
       <c r="J16" s="3" t="n"/>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Phân biệt việc cập nhật chuỗi đầu vào với việc cập nhật trọng số của mô hình.</t>
+          <t>Trong mô hình tự hồi quy (autoregressive language model), sau khi chọn token 'mưa', token này được nối trực tiếp vào chuỗi ngữ cảnh đầu vào (context) để làm đầu vào cho lượt dự đoán token kế tiếp.</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I17" s="4" t="n">
         <v>60</v>
@@ -1375,7 +1375,7 @@
       <c r="J17" s="3" t="n"/>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Dung lượng ngữ cảnh được tính theo token của cách biểu diễn dữ liệu, không theo ý nghĩa trừu tượng.</t>
+          <t>JSON tốn 820 token trong khi Bảng rút gọn tốn 510 token cho cùng thông tin, do đó Bảng rút gọn tiết kiệm 820 - 510 = 310 token ngữ cảnh cho mỗi lần gửi.</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2,4</t>
+          <t>1,2,3,5</t>
         </is>
       </c>
       <c r="I18" s="4" t="n">
@@ -1428,7 +1428,7 @@
       <c r="J18" s="3" t="n"/>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Chỉ xét những đặc trưng thực sự nằm trong chuỗi đầu vào của tokenizer.</t>
+          <t>Các yếu tố trong chuỗi đầu vào làm thay đổi số token gồm: Ngôn ngữ và vốn từ tokenizer đã học (a), Dấu câu và khoảng trắng (b), Ký hiệu cú pháp cấu trúc như JSON/code (c), và Thuật toán tách mảnh từ (e). Màu nền của editor (d) không được gửi vào tokenizer nên không ảnh hưởng.</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1472,7 @@
       </c>
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I19" s="4" t="n">
         <v>60</v>
@@ -1480,7 +1480,7 @@
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: So sánh đơn vị mà `split()` đếm với đơn vị mà mô hình xử lý.</t>
+          <t>Dùng `tokenizer.encode()` chính xác hơn `len(text.split())` vì tokenizer sử dụng đúng từ điển và thuật toán tách mảnh từ (BPE/WordPiece) của mô hình, đếm chính xác số đơn vị token mà mô hình thực sự nhận.</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I21" s="4" t="n">
         <v>60</v>
@@ -1572,7 +1572,7 @@
       <c r="J21" s="3" t="n"/>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: So sánh nhóm nào có kết quả đa dạng hơn dựa trên đầu ra quan sát được.</t>
+          <t>Khi chỉ temperature thay đổi, nhóm Y đa dạng hơn và có câu lạc đề chứng tỏ nhóm Y được chạy với temperature cao hơn nhóm X (temperature cao làm phẳng phân phối xác suất và tăng tính ngẫu nhiên).</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>2,4</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="I23" s="4" t="n">
@@ -1685,7 +1685,7 @@
       <c r="J23" s="3" t="n"/>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Dừng ở token làm tổng xác suất tích lũy lần đầu đạt hoặc vượt ngưỡng.</t>
+          <t>Các token sắp xếp giảm dần: K = 0,50; L = 0,20; M = 0,15... Với top-p = 0,68, tổng tích lũy: K = 0,50 (&lt; 0,68); K + L = 0,70 (&gt;= 0,68). Vậy tập nhỏ nhất được giữ lại gồm {K, L}.</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I24" s="4" t="n">
         <v>60</v>
@@ -1731,7 +1731,7 @@
       <c r="J24" s="3" t="n"/>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Hình dung tổng xác suất tích lũy sẽ đạt ngưỡng sớm hay muộn khi top-p nhỏ đi.</t>
+          <t>Khi giảm top-p từ 0,95 xuống 0,60, tổng xác suất tích lũy của các token có xác suất cao nhất đạt ngưỡng 0,60 sớm hơn, khiến tập token ứng viên được giữ lại trở nên hẹp hơn.</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -1777,7 +1777,7 @@
       <c r="J25" s="3" t="n"/>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Chia ngân sách đầu ra cho số bản tóm tắt độc lập.</t>
+          <t>Ngân sách tối đa 2.400 token đầu ra chia đều cho 12 bản tóm tắt độc lập: 2.400 / 12 = 200 token cho mỗi bản.</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="G26" s="3" t="n"/>
       <c r="H26" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I26" s="4" t="n">
         <v>60</v>
@@ -1823,7 +1823,7 @@
       <c r="J26" s="3" t="n"/>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Phân biệt cấu hình trước khi gọi với thông tin cho biết lý do dừng sau khi nhận phản hồi.</t>
+          <t>Khi đặt `max_output_tokens=120` và phản hồi bị dừng giữa câu, có thể mô hình đã chạm giới hạn đầu ra; cần kiểm tra `finish_reason` trong phản hồi (nếu là 'length' thì khẳng định bị cắt do hết token).</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3000</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -1915,7 +1915,7 @@
       <c r="J28" s="3" t="n"/>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Cộng mọi thành phần trước rồi lấy dung lượng cửa sổ trừ đi tổng đó.</t>
+          <t>Tổng số token đã phân bổ gồm lời nhắc (2.500), lịch sử hội thoại (8.500), ngữ cảnh truy xuất (12.000) và giới hạn đầu ra (6.000) là: 2.500 + 8.500 + 12.000 + 6.000 = 29.000 token. Số token còn dư trong cửa sổ ngữ cảnh 32.000 là: 32.000 - 29.000 = 3.000 token.</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="G29" s="3" t="n"/>
       <c r="H29" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I29" s="4" t="n">
         <v>60</v>
@@ -1968,7 +1968,7 @@
       <c r="J29" s="3" t="n"/>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tính phần vượt trước, rồi loại các phương án làm mất phần bằng chứng phải giữ.</t>
+          <t>Tổng ngân sách hiện tại = 2.000 (prompt) + 6.000 (history) + 7.000 (evidence) + 4.000 (output) = 19.000 token, vượt cửa sổ 16.000 là 3.000 token. Giảm giới hạn đầu ra 2.000 token và tóm tắt giảm lịch sử 1.000 token giúp giảm đúng 3.000 token vừa vặn cửa sổ mà vẫn giữ nguyên bằng chứng 7.000.</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="G31" s="3" t="n"/>
       <c r="H31" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I31" s="4" t="n">
         <v>60</v>
@@ -2060,7 +2060,7 @@
       <c r="J31" s="3" t="n"/>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tìm dấu hiệu cho thấy câu trả lời có thể đã thay đổi sau thời điểm mô hình được huấn luyện.</t>
+          <t>Giá API và endpoint thay đổi theo thời gian thực và không thể trả lời chính xác từ trí nhớ tĩnh của mô hình; cách xử lý đúng là tra cứu tài liệu chính thức hiện hành hoặc gọi tool tìm kiếm và ghi rõ mốc thời gian kiểm tra.</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>1-A, 2-B, 3-C</t>
+          <t>1-B, 2-C, 3-A</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2168,7 +2168,7 @@
       <c r="J33" s="3" t="n"/>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tìm đơn vị rời rạc hoặc từng đoạn mà mô hình xử lý sau bước tiền xử lý.</t>
+          <t>Văn bản (x1) biểu diễn bằng mảnh từ hoặc mã định danh token (r1); Hình ảnh (x2) biểu diễn bằng mảnh ảnh (image patches) hoặc token hình ảnh (r2); Âm thanh (x3) biểu diễn bằng khung/đoạn âm thanh được mã hóa thành token (r3).</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="G35" s="3" t="n"/>
       <c r="H35" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I35" s="4" t="n">
         <v>60</v>
@@ -2270,7 +2270,7 @@
       <c r="J35" s="3" t="n"/>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Giữ kết luận trong đúng phạm vi và đúng loại cơ chế đã được đo.</t>
+          <t>Các thí nghiệm probe và can thiệp trên mô hình Othello chỉ chứng minh mô hình học được biểu diễn nội tại về trạng thái bàn cờ của trò chơi đó. Kết luận 'Mô hình đã có hiểu biết có ý thức và world model tổng quát cho mọi lĩnh vực' vượt quá bằng chứng thu được nhiều nhất.</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I37" s="4" t="n">
         <v>60</v>
@@ -2362,7 +2362,7 @@
       <c r="J37" s="3" t="n"/>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Cùng danh tính token nhưng vai trò có thể thay đổi theo vị trí trong câu.</t>
+          <t>Kiến trúc Transformer xử lý các token song song và có tính bất biến với thứ tự (permutation invariant); positional encoding bổ sung thông tin vị trí vào vector biểu diễn để attention phân biệt được trật tự từ ('chó cắn mèo' khác 'mèo cắn chó').</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>o1 → o2 → o3 → o4</t>
+          <t>o4 → o2 → o1 → o3</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -2414,7 +2414,7 @@
       <c r="J38" s="3" t="n"/>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Attention cần nhận biểu diễn đã mang cả danh tính token và vị trí.</t>
+          <t>Luồng đầu vào Transformer trước khối attention gồm: tách văn bản thành token IDs (o4) -&gt; tra token embedding từ token IDs (o2) -&gt; cộng hoặc kết hợp thông tin vị trí positional encoding (o1) -&gt; đưa biểu diễn vào khối attention (o3).</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2554,7 @@
       </c>
       <c r="G41" s="3" t="n"/>
       <c r="H41" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I41" s="4" t="n">
         <v>60</v>
@@ -2562,7 +2562,7 @@
       <c r="J41" s="3" t="n"/>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Giữ kết luận trong đúng head, đúng tầng và đúng ba token được quan sát.</t>
+          <t>Trọng số attention 0,62 tới `river` cho thấy trong head và tầng cụ thể này, biểu diễn của token `bank` nhận được đóng góp lớn nhất từ token `river` trong số ba token được quan sát.</t>
         </is>
       </c>
     </row>
@@ -2649,7 +2649,7 @@
       </c>
       <c r="G43" s="3" t="n"/>
       <c r="H43" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I43" s="4" t="n">
         <v>60</v>
@@ -2657,7 +2657,7 @@
       <c r="J43" s="3" t="n"/>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: So sánh dữ liệu có sẵn ở bước huấn luyện với dữ liệu thật sự có khi sinh tuần tự.</t>
+          <t>Khi dự đoán token ở vị trí 5, việc che token ở vị trí 6 (causal mask) là bắt buộc vì nếu cho phép nhìn thấy vị trí 6, mô hình sẽ bị rò rỉ thông tin tương lai - điều không thể xảy ra khi sinh văn bản tự hồi quy ở thời điểm suy luận.</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="G44" s="3" t="n"/>
       <c r="H44" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I44" s="4" t="n">
         <v>60</v>
@@ -2703,7 +2703,7 @@
       <c r="J44" s="3" t="n"/>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: So sánh từng chỉ số key với chỉ số query.</t>
+          <t>Trong decoder nhân quả, query tại vị trí 3 chỉ được phép chú ý tới các key tại vị trí &lt;= 3. Việc mask cho phép key 4 làm rò rỉ thông tin tương lai vào bước suy luận hiện tại.</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="G47" s="3" t="n"/>
       <c r="H47" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I47" s="4" t="n">
         <v>60</v>
@@ -2847,7 +2847,7 @@
       <c r="J47" s="3" t="n"/>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Residual nghĩa là giữ một đường đi tắt của biểu diễn trước tầng biến đổi.</t>
+          <t>Đường kết nối tắt residual (residual skip connection) quanh khối attention nhận đầu vào ban đầu `x` và cộng trực tiếp với đầu ra của tầng `Attention(x)`, tạo thành `x + Attention(x)` trước khi đi vào LayerNorm.</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>o1 → o2 → o3 → o4</t>
+          <t>o2 → o4 → o1 → o3</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -2904,7 +2904,7 @@
       <c r="J48" s="3" t="n"/>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Theo dõi biến nào phải được tạo trước khi xuất hiện ở vế phải.</t>
+          <t>Thứ tự qua khối Transformer (Post-Norm): attention tính a = Attention(x) (o2) -&gt; residual &amp; norm tính r1 = Norm(x + a) (o4) -&gt; feed-forward tính f = FFN(r1) (o1) -&gt; residual &amp; norm thứ hai tính r2 = Norm(r1 + f) (o3).</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>1-A, 2-B, 3-C</t>
+          <t>1-C, 2-B, 3-A</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -2960,7 +2960,7 @@
       <c r="J49" s="3" t="n"/>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tách chuỗi nguồn khỏi tiền tố token đích, rồi hỏi đường nào nối hai phía.</t>
+          <t>Self-attention của encoder (x1) truy cập các vị trí nguồn trong đầu vào encoder (r1); Causal self-attention của decoder (x2) truy cập các vị trí token đích hiện tại hoặc quá khứ (r2); Cross-attention của decoder (x3) truy cập đầu ra encoder khi decoder sinh token đích (r3).</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="G50" s="3" t="n"/>
       <c r="H50" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I50" s="4" t="n">
         <v>60</v>
@@ -3006,7 +3006,7 @@
       <c r="J50" s="3" t="n"/>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Kiểm tra có hai ngăn xếp nguồn/đích và cross-attention, hay chỉ một ngăn xếp nhân quả.</t>
+          <t>Mô hình nhận lời nhắc trong cùng một chuỗi và sinh token tiếp theo theo kiểu tự hồi quy mà không có encoder riêng hay cross-attention thuộc họ kiến trúc Transformer chỉ có decoder (Decoder-only Transformer, như GPT, LLaMA).</t>
         </is>
       </c>
     </row>
@@ -3104,7 +3104,7 @@
       </c>
       <c r="G52" s="3" t="n"/>
       <c r="H52" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I52" s="4" t="n">
         <v>60</v>
@@ -3112,7 +3112,7 @@
       <c r="J52" s="3" t="n"/>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Dữ liệu không chỉ có một câu trả lời đích; nó so sánh hai câu trả lời.</t>
+          <t>Tập dữ liệu gồm chỉ dẫn, hai câu trả lời A/B và nhãn người đánh giá thích A hơn B là dữ liệu so sánh ưu tiên trực tiếp phục vụ giai đoạn căn chỉnh theo ưu tiên (preference alignment, như RLHF hoặc DPO).</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>1-A, 2-B, 3-C, 4-D</t>
+          <t>1-B, 2-A, 3-C, 4-D</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -3224,7 +3224,7 @@
       <c r="J54" s="3" t="n"/>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Phân biệt dữ liệu giám sát, mô hình chấm điểm và mô hình sinh câu trả lời.</t>
+          <t>Câu trả lời mẫu do con người viết (x1) là đích giám sát cho hành vi ban đầu (SFT target) (r1); Nhãn ưu tiên A hơn B (x2) là tín hiệu xếp hạng các câu trả lời (r2); Mô hình thưởng (x3) ước lượng điểm thưởng cho câu trả lời (r3); Mô hình chính sách policy (x4) là mô hình sinh câu trả lời được tối ưu (r4).</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="G56" s="3" t="n"/>
       <c r="H56" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I56" s="4" t="n">
         <v>60</v>
@@ -3322,7 +3322,7 @@
       <c r="J56" s="3" t="n"/>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tìm pipeline không có bước huấn luyện reward model riêng và vòng lặp tối ưu policy bằng RL.</t>
+          <t>Phương pháp tối ưu policy trực tiếp từ các cặp câu trả lời ưu tiên với một policy tham chiếu mà không cần huấn luyện reward model riêng hay chạy thuật toán RL là DPO (Direct Preference Optimization).</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3370,7 @@
       </c>
       <c r="H57" s="4" t="inlineStr">
         <is>
-          <t>2,3</t>
+          <t>1,2</t>
         </is>
       </c>
       <c r="I57" s="4" t="n">
@@ -3379,7 +3379,7 @@
       <c r="J57" s="3" t="n"/>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Đừng loại bỏ các cặp ưu tiên chỉ vì phương pháp này được gọi là trực tiếp.</t>
+          <t>DPO tối ưu trực tiếp policy từ dữ liệu ưu tiên thông qua hàm mất mát dạng phân loại nhị phân, do đó không cần giai đoạn huấn luyện reward model riêng (a) và không cần vòng lặp học tăng cường PPO (b).</t>
         </is>
       </c>
     </row>
@@ -3419,7 +3419,7 @@
       </c>
       <c r="G58" s="3" t="n"/>
       <c r="H58" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I58" s="4" t="n">
         <v>60</v>
@@ -3427,7 +3427,7 @@
       <c r="J58" s="3" t="n"/>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Giữ phạm vi đối tượng và nhiệm vụ trong kết luận trùng với phạm vi của bài đánh giá.</t>
+          <t>Đạt 99% trên một bài đánh giá an toàn cố định chỉ chứng minh mô hình có hiệu năng cao trên phân phối của bài đánh giá đó; trong thực tế triển khai, mô hình vẫn cần được kiểm thử trên các phân phối và kiểu tấn công đối kháng khác.</t>
         </is>
       </c>
     </row>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="H59" s="4" t="inlineStr">
         <is>
-          <t>2,4</t>
+          <t>1,2,3,5</t>
         </is>
       </c>
       <c r="I59" s="4" t="n">
@@ -3482,7 +3482,7 @@
       <c r="J59" s="3" t="n"/>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Chọn bằng chứng quan sát hành vi trong nhiều điều kiện; đừng coi tên thuật toán là bảo chứng.</t>
+          <t>Đánh giá an toàn toàn diện cần: Red-team bằng lời nhắc đối kháng (a), Đánh giá trên phân phối thực tế (b), Theo dõi dạng lỗi và độ không chắc chắn (c), và Kiểm tra mức tuân thủ chính sách theo rubric (e). Chỉ biết tên phương pháp (d) không phải là bằng chứng kiểm chứng.</t>
         </is>
       </c>
     </row>
@@ -3510,7 +3510,7 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>1-A, 2-B, 3-C</t>
+          <t>1-C, 2-B, 3-A</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -3538,7 +3538,7 @@
       <c r="J60" s="3" t="n"/>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Hỏi thay đổi xảy ra trước mô hình nền, sau mô hình nền hay trong lúc suy luận.</t>
+          <t>Tăng kho dữ liệu và năng lực tính toán cho việc dự đoán token kế tiếp (x1) thuộc Tiền huấn luyện pre-training (r1); Tinh chỉnh theo chỉ dẫn/ưu tiên sau khi có base model (x2) thuộc Hậu huấn luyện post-training (r2); Giữ nguyên trọng số, thực hiện thêm nhiều bước suy luận/tìm kiếm khi trả lời (x3) thuộc Tính toán tại thời điểm suy luận test-time compute (r3).</t>
         </is>
       </c>
     </row>
@@ -3560,7 +3560,7 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0.48</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -3588,7 +3588,7 @@
       <c r="J61" s="3" t="n"/>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tính token đầu vào và đầu ra riêng theo đúng đơn giá, rồi mới cộng hai khoản.</t>
+          <t>Chi phí token đầu vào = 120.000 × (2 USD / 1.000.000) = 0,24 USD. Chi phí token đầu ra = 30.000 × (8 USD / 1.000.000) = 0,24 USD. Tổng chi phí là 0,24 + 0,24 = 0,48 USD.</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0.06</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -3638,7 +3638,7 @@
       <c r="J62" s="3" t="n"/>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tính tổng chi phí của từng nhà cung cấp bằng hai đơn giá riêng, rồi lấy chi phí của B trừ chi phí của A.</t>
+          <t>Chi phí tại Nhà cung cấp A = (800.000 × 0,50 + 200.000 × 1,50) / 1.000.000 = 0,40 + 0,30 = 0,70 USD. Chi phí tại Nhà cung cấp B = (800.000 × 0,70 + 200.000 × 1,00) / 1.000.000 = 0,56 + 0,20 = 0,76 USD. Chênh lệch chi phí: B − A = 0,76 − 0,70 = 0,06 USD (A rẻ hơn B 0,06 USD).</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1.05</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -3689,7 +3689,7 @@
       <c r="J63" s="3" t="n"/>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Nhân số token của một request với 50 trước, rồi áp riêng hai đơn giá.</t>
+          <t>Tổng số token đầu vào cả lô = 50 × 4.000 = 200.000 token, chi phí đầu vào = 200.000 × (3 / 1.000.000) = 0,60 USD. Tổng số token đầu ra cả lô = 50 × 1.000 = 50.000 token, chi phí đầu ra = 50.000 × (9 / 1.000.000) = 0,45 USD. Tổng chi phí toàn bộ lô = 0,60 + 0,45 = 1,05 USD.</t>
         </is>
       </c>
     </row>
@@ -3711,7 +3711,7 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6600</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -3739,7 +3739,7 @@
       <c r="J64" s="3" t="n"/>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Hạch toán từng request riêng; phần lịch sử được gửi lại vẫn được tính trong request mới.</t>
+          <t>Tổng số token đầu vào qua ba lượt = 1.000 + 1.800 + 2.600 = 5.400 token. Tổng số token đầu ra qua ba lượt = 3 × 400 = 1.200 token. Tổng số token được hạch toán là 5.400 + 1.200 = 6.600 token.</t>
         </is>
       </c>
     </row>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="H65" s="4" t="inlineStr">
         <is>
-          <t>1,5</t>
+          <t>1,2,4</t>
         </is>
       </c>
       <c r="I65" s="4" t="n">
@@ -3792,7 +3792,7 @@
       <c r="J65" s="3" t="n"/>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Giảm phần lặp không liên quan, nhưng không được xóa mù quáng dữ kiện bắt buộc.</t>
+          <t>Các biện pháp giảm chi phí token lặp lại hợp lý: Tóm tắt có kiểm soát lịch sử cũ (a), Chỉ truy xuất đoạn tài liệu liên quan cho từng request (b), và Giới hạn số lượt lịch sử giữ nguyên văn (d). Giữ nguyên toàn bộ nhật ký (c) không giảm chi phí, còn lược bỏ chỉ dẫn bắt buộc (e) làm hỏng chất lượng.</t>
         </is>
       </c>
     </row>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="G66" s="3" t="n"/>
       <c r="H66" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I66" s="4" t="n">
         <v>60</v>
@@ -3846,7 +3846,7 @@
       <c r="J66" s="3" t="n"/>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Loại hồ sơ vi phạm giới hạn bắt buộc về ngữ cảnh trước khi so sánh chi phí và chất lượng.</t>
+          <t>Hợp đồng có 90k token đầu vào và 8k token đầu ra (tổng 98k token), vượt giới hạn 32k của Tier S, trong khi Tier L quá đắt vượt ngân sách hạn chế. Do đó Tier M với ngữ cảnh 128k và chi phí vừa phải là lựa chọn phù hợp nhất.</t>
         </is>
       </c>
     </row>
@@ -3949,7 +3949,7 @@
       </c>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>3,4</t>
+          <t>1,2,3,4</t>
         </is>
       </c>
       <c r="I68" s="4" t="n">
@@ -3958,7 +3958,7 @@
       <c r="J68" s="3" t="n"/>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Giữ mọi yếu tố ngoài danh tính model càng nhất quán càng tốt.</t>
+          <t>Trong thí nghiệm so sánh hai mô hình, mọi yếu tố ngoài danh tính mô hình (e) đều là biến gây nhiễu cần chuẩn hóa: Prompt và ngôn ngữ khác nhau (a), Temperature khác nhau (b), Chỉ chạy 1 lần không đo được phương sai (c), và Ranh giới đo độ trễ khác nhau (d).</t>
         </is>
       </c>
     </row>
@@ -4002,7 +4002,7 @@
       </c>
       <c r="H69" s="4" t="inlineStr">
         <is>
-          <t>1,3</t>
+          <t>1,2,3,4</t>
         </is>
       </c>
       <c r="I69" s="4" t="n">
@@ -4011,7 +4011,7 @@
       <c r="J69" s="3" t="n"/>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Giữ đủ dữ liệu để người khác tái lập lý do một model được chọn.</t>
+          <t>Để tái lập và kiểm tra lại phép so sánh model, schema kết quả cần ghi nhận: ID mô hình và case_id/prompt (a), Các tham số sinh như temperature, top_p (b), Đầu ra thô và điểm số theo rubric (c), cùng Độ trễ và số token sử dụng (d).</t>
         </is>
       </c>
     </row>
@@ -4041,7 +4041,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>1-A, 2-B, 3-C, 4-D</t>
+          <t>1-C, 2-B, 3-D, 4-A</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -4069,7 +4069,7 @@
       <c r="J70" s="3" t="n"/>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Hỏi ai gọi model, qua giao diện nào và ai chịu trách nhiệm về hạ tầng.</t>
+          <t>Cá nhân hỏi đáp thủ công, không cần tích hợp (x1) dùng Giao diện trò chuyện Chat UI (r1); IDE cần gợi ý code theo repository (x2) dùng Trợ lý lập trình coding assistant (r2); Phần backend gọi model theo từng request (x3) dùng API do nhà cung cấp vận hành hosted API (r3); Tổ chức giữ trọng số và suy luận trong hạ tầng riêng (x4) dùng Tự vận hành self-hosted (r4).</t>
         </is>
       </c>
     </row>
@@ -4109,7 +4109,7 @@
       </c>
       <c r="G71" s="3" t="n"/>
       <c r="H71" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I71" s="4" t="n">
         <v>60</v>
@@ -4117,7 +4117,7 @@
       <c r="J71" s="3" t="n"/>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Chọn giao diện đáp ứng trường hợp sử dụng hiện tại, không tối ưu cho nhu cầu chưa có.</t>
+          <t>Khi chỉ cần thử nghiệm ý tưởng trong 30 phút bằng vài prompt thủ công mà chưa cần viết code hay tích hợp, Giao diện trò chuyện (Chat UI) là chế độ có chi phí chuẩn bị thấp nhất và nhanh nhất.</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="G72" s="3" t="n"/>
       <c r="H72" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I72" s="4" t="n">
         <v>60</v>
@@ -4165,7 +4165,7 @@
       <c r="J72" s="3" t="n"/>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Chỉ kết luận thuộc tính được đo trực tiếp; hãy liệt kê các siêu dữ liệu còn thiếu.</t>
+          <t>Con số công bố `Model X: 300B total parameters` chỉ cho biết quy mô tổng số tham số; nếu là kiến trúc MoE (Mixture of Experts) thì số tham số hoạt động ở mỗi token thấp hơn nhiều, nên chưa đủ dữ kiện để suy ra năng lực tính toán mỗi token hay độ trễ phục vụ.</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
       </c>
       <c r="G73" s="3" t="n"/>
       <c r="H73" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I73" s="4" t="n">
         <v>60</v>
@@ -4213,7 +4213,7 @@
       <c r="J73" s="3" t="n"/>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Áp dụng ngưỡng trước, rồi mới tối ưu chỉ số phụ như chi phí.</t>
+          <t>Tiêu chí ưu tiên hàng đầu là độ chính xác thực tế với ngưỡng bắt buộc 92%. Model F chỉ đạt 88% nên bị loại trực tiếp; Model E đạt 94% vượt ngưỡng nên được chọn dù chi phí cao hơn.</t>
         </is>
       </c>
     </row>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="H75" s="4" t="inlineStr">
         <is>
-          <t>1,3</t>
+          <t>1,2,3,5</t>
         </is>
       </c>
       <c r="I75" s="4" t="n">
@@ -4319,7 +4319,7 @@
       <c r="J75" s="3" t="n"/>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Phân biệt file cấu hình mẫu với file chứa credential thật, rồi kiểm tra cách xử lý khi biến môi trường không tồn tại.</t>
+          <t>Thực hành an toàn cấu hình: Xóa secret hard-code khỏi source (a), Bỏ track .env và thêm vào .gitignore (b), Giữ .env.example mẫu không có secret thật (c), và Báo lỗi cấu hình rõ ràng trước khi gọi mạng (e). In key ra log (d) là lỗ hổng rò rỉ credential.</t>
         </is>
       </c>
     </row>
@@ -4357,7 +4357,7 @@
       </c>
       <c r="G76" s="3" t="n"/>
       <c r="H76" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I76" s="4" t="n">
         <v>60</v>
@@ -4365,7 +4365,7 @@
       <c r="J76" s="3" t="n"/>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tách lỗi cấu hình cục bộ khỏi lỗi do server trả sau lời gọi mạng.</t>
+          <t>Khi `os.getenv('API_KEY')` trả về `None`, cách xử lý đúng là kiểm tra ngay sau khi nạp cấu hình và ném lỗi rõ ràng trước khi thực hiện network call, thay vì gửi đi request lỗi xác thực mơ hồ.</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="G77" s="3" t="n"/>
       <c r="H77" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I77" s="4" t="n">
         <v>60</v>
@@ -4419,7 +4419,7 @@
       <c r="J77" s="3" t="n"/>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Đối chiếu từng trường với chữ ký hàm được cung cấp; không dùng trí nhớ về SDK khác.</t>
+          <t>Lệnh gọi đúng contract phải truyền đúng các trường: model='m1', messages gồm system message trước rồi đến user message, temperature=0.2 và max_output_tokens=200.</t>
         </is>
       </c>
     </row>
@@ -4484,7 +4484,7 @@
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
-          <t>3,5</t>
+          <t>1,2,3,5</t>
         </is>
       </c>
       <c r="I78" s="4" t="n">
@@ -4493,7 +4493,7 @@
       <c r="J78" s="3" t="n"/>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: So cả tên trường lẫn ý nghĩa/giá trị được đặt vào trường đó.</t>
+          <t>Lệnh gọi bị các lỗi: Đặt nhầm content vào role đối nghịch (a), Message order đưa user trước system (b), Tráo giá trị temperature=200 và max_tokens=0.2 (c), trong khi tên phương thức `client.chat.create` vẫn đúng contract (e).</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="G79" s="3" t="n"/>
       <c r="H79" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I79" s="4" t="n">
         <v>60</v>
@@ -4539,7 +4539,7 @@
       <c r="J79" s="3" t="n"/>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Đi theo cấu trúc choice → message → content.</t>
+          <t>Cấu trúc phản hồi là dict lồng nhau: để lấy văn bản được sinh từ `{'choices':[{'message':{'content':'Xin chào'}}]}`, biểu thức truy xuất chính xác là `response['choices'][0]['message']['content']`.</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="G81" s="3" t="n"/>
       <c r="H81" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I81" s="4" t="n">
         <v>60</v>
@@ -4631,7 +4631,7 @@
       <c r="J81" s="3" t="n"/>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tên có chữ `output` không đồng nghĩa trường đó chứa văn bản output.</t>
+          <t>Các trường `input_tokens=80`, `output_tokens=20` và `total_tokens=100` đều là các trường số liệu thống kê việc sử dụng token (usage metrics) của request, không chứa nội dung văn bản.</t>
         </is>
       </c>
     </row>
@@ -4659,7 +4659,7 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>1-A, 2-B, 3-C</t>
+          <t>1-A, 2-C, 3-B</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -4687,7 +4687,7 @@
       <c r="J82" s="3" t="n"/>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Một `finish_reason` nói về kết thúc bình thường, một về giới hạn output, một về chuyển quyền thực thi hành động.</t>
+          <t>stop (x1) là kết thúc bình thường theo điều kiện dừng (r1); length (x2) là bị cắt do chạm giới hạn token (r2); tool_call (x3) là chuyển sang thực thi/phân phối tool theo contract (r3).</t>
         </is>
       </c>
     </row>
@@ -4725,7 +4725,7 @@
       </c>
       <c r="G83" s="3" t="n"/>
       <c r="H83" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I83" s="4" t="n">
         <v>60</v>
@@ -4733,7 +4733,7 @@
       <c r="J83" s="3" t="n"/>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Hãy ưu tiên metadata thay vì đoán chỉ từ dấu câu cuối.</t>
+          <t>Khi `finish_reason='length'`, câu trả lời chưa kết thúc tự nhiên mà bị cắt do chạm trần token. Ứng dụng phải đánh dấu bị cắt, không trình bày như câu trả lời hoàn chỉnh, và thực hiện retry có điều chỉnh tăng giới hạn token hoặc yêu cầu viết tiếp có kiểm soát.</t>
         </is>
       </c>
     </row>
@@ -4771,7 +4771,7 @@
       </c>
       <c r="G84" s="3" t="n"/>
       <c r="H84" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I84" s="4" t="n">
         <v>60</v>
@@ -4779,7 +4779,7 @@
       <c r="J84" s="3" t="n"/>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Bắt đầu ngay trước lời gọi mạng và kết thúc ngay sau khi lời gọi trả về.</t>
+          <t>Để đo độ trễ thuần của lời gọi API, mốc thời gian bắt đầu `start=now()` phải đặt ngay trước lời gọi mạng `response=client.call(req)` và mốc kết thúc tính ngay sau khi lời gọi trả về `elapsed=now()-start`, không kèm bước nạp dữ liệu hay render.</t>
         </is>
       </c>
     </row>
@@ -4797,7 +4797,7 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1.575</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -4825,7 +4825,7 @@
       <c r="J85" s="3" t="n"/>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Thời gian trôi qua = thời điểm kết thúc − thời điểm bắt đầu.</t>
+          <t>Độ trễ thuần của lời gọi API = Thời điểm kết thúc − Thời điểm bắt đầu = 13,925 − 12,350 = 1,575 giây.</t>
         </is>
       </c>
     </row>
@@ -4853,7 +4853,7 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>1-A, 2-B, 3-C</t>
+          <t>1-B, 2-A, 3-C</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
@@ -4881,7 +4881,7 @@
       <c r="J86" s="3" t="n"/>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Hỏi instruction nào phải giữ nguyên qua nhiều task của user.</t>
+          <t>'Luôn trả lời như trợ giảng, không tiết lộ secret' (x1) là System content (r1); 'Hãy giải thích attention cho tôi bằng ví dụ' (x2) là User content (r2); 'System message phải xuất hiện trước user message' (x3) là Ràng buộc thứ tự, không phải nội dung yêu cầu của người học (r3).</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>1-A, 2-B, 3-C, 4-D</t>
+          <t>1-C, 2-B, 3-D, 4-A</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
@@ -4939,7 +4939,7 @@
       <c r="J87" s="3" t="n"/>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Mỗi lớp trả lời một câu: model hành xử ra sao, user muốn gì, dùng dữ kiện nào và output phải có dạng gì.</t>
+          <t>'Bạn là chuyên viên phân tích...' (x1) là Chỉ dẫn system về cách model hành xử (r1); 'Câu hỏi: Vì sao doanh thu giảm?' (x2) là Input hiện tại của user (r2); 'Bảng doanh thu Q1–Q4' (x3) là Context hỗ trợ (r3); 'Trả JSON gồm cause và evidence_row' (x4) là Hợp đồng output (r4).</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5077,7 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>1-A, 2-B, 3-C</t>
+          <t>1-A, 2-C, 3-B</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
@@ -5105,7 +5105,7 @@
       <c r="J90" s="3" t="n"/>
       <c r="K90" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Tách đường dẫn content khỏi hai trường thống kê token.</t>
+          <t>choices[0].message.content (x1) tương ứng với result.text (r1); usage.prompt_tokens (x2) tương ứng với metrics.input_tokens (r2); usage.completion_tokens (x3) tương ứng với metrics.output_tokens (r3).</t>
         </is>
       </c>
     </row>
@@ -5129,7 +5129,7 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>o1 → o2 → o3 → o4</t>
+          <t>o2 → o3 → o4 → o1</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -5157,7 +5157,7 @@
       <c r="J91" s="3" t="n"/>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Theo dõi kiểu dữ liệu: text → token ID/tensor → ID được sinh → text.</t>
+          <t>Quy trình suy luận causal language model cục bộ: Nạp tokenizer và causal LM tương thích (o2) -&gt; Tokenize/encode prompt thành tensor (o3) -&gt; Gọi generate với giới hạn output (o4) -&gt; Giải mã (decode) các token ID được sinh thành text (o1).</t>
         </is>
       </c>
     </row>
@@ -5195,7 +5195,7 @@
       </c>
       <c r="G92" s="3" t="n"/>
       <c r="H92" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I92" s="4" t="n">
         <v>60</v>
@@ -5203,7 +5203,7 @@
       <c r="J92" s="3" t="n"/>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Token ID chỉ có ý nghĩa trong vocabulary mà model đã được huấn luyện.</t>
+          <t>Nạp tokenizer của `model-A` nhưng nạp trọng số của `model-B` khi từ điển khác nhau sẽ dẫn đến việc các token ID bị ánh xạ sai lệch hoàn toàn hoặc vượt quá phạm vi embedding matrix của model, gây lỗi crash hoặc sinh rác.</t>
         </is>
       </c>
     </row>
@@ -5241,7 +5241,7 @@
       </c>
       <c r="G93" s="3" t="n"/>
       <c r="H93" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I93" s="4" t="n">
         <v>60</v>
@@ -5249,7 +5249,7 @@
       <c r="J93" s="3" t="n"/>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Phân biệt đối tượng truyền tải với từng phần dữ liệu nội dung.</t>
+          <t>Khi một hàm trả về stream (iterator các chunk/event) trong khi bên gọi cần chuỗi hoàn chỉnh, lỗi là iterator chưa được duyệt và các delta nội dung chưa được trích xuất để ghép nối lại thành một chuỗi text hoàn chỉnh.</t>
         </is>
       </c>
     </row>
@@ -5272,7 +5272,7 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>o1 → o2 → o3</t>
+          <t>o2 → o3 → o1</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
@@ -5300,7 +5300,7 @@
       <c r="J94" s="3" t="n"/>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Dùng số thứ tự, không dùng thứ tự các phần tử đến.</t>
+          <t>Khi các delta đến lệch thứ tự (3,'C'), (1,'A'), (2,'B'), hợp đồng yêu cầu phát theo số thứ tự: Thứ tự 1: A (o2) -&gt; Thứ tự 2: B (o3) -&gt; Thứ tự 3: C (o1).</t>
         </is>
       </c>
     </row>
@@ -5328,7 +5328,7 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>1-A, 2-B, 3-C</t>
+          <t>1-B, 2-C, 3-A</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -5356,7 +5356,7 @@
       <c r="J95" s="3" t="n"/>
       <c r="K95" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Hỏi kết quả từng phần có an toàn và hữu ích trước khi hoàn tất hay không.</t>
+          <t>Cuộc trò chuyện dài, người dùng chấp nhận đọc dần (x1) dùng truyền kết quả từng phần streaming (r1); JSON phải kiểm tra toàn bộ trước khi hệ thống tài chính nhận (x2) cần giữ toàn bộ kết quả rồi kiểm tra trước khi chuyển tiếp (r2); Xử lý theo lô ở chế độ ngoại tuyến không người chờ (x3) dùng thu thập theo lô đơn giản (r3).</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5394,7 @@
       </c>
       <c r="G96" s="3" t="n"/>
       <c r="H96" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I96" s="4" t="n">
         <v>60</v>
@@ -5402,7 +5402,7 @@
       <c r="J96" s="3" t="n"/>
       <c r="K96" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Ràng buộc quyết định là `trước khi hiển thị bất kỳ byte nào`.</t>
+          <t>Nếu ứng dụng có yêu cầu bắt buộc phải kiểm tra schema và chữ ký trên toàn bộ phản hồi trước khi hiển thị bất kỳ byte nào, chế độ phù hợp trực tiếp là không streaming hoặc phải đệm (buffer) toàn bộ response rồi mới hiển thị.</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>o1 → o2 → o3 → o4</t>
+          <t>o2 → o3 → o4 → o1</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
@@ -5454,7 +5454,7 @@
       <c r="J97" s="3" t="n"/>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Mỗi câu trả lời của assistant phải đứng sau lượt user mà nó trả lời.</t>
+          <t>Thứ tự hội thoại theo thời gian bắt đầu từ trạng thái rỗng là: user:U1 (o2) -&gt; assistant:A1 (o3) -&gt; user:U2 (o4) -&gt; assistant:A2 (o1).</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5498,7 @@
       </c>
       <c r="H98" s="4" t="inlineStr">
         <is>
-          <t>2,3</t>
+          <t>1,2,3</t>
         </is>
       </c>
       <c r="I98" s="4" t="n">
@@ -5507,7 +5507,7 @@
       <c r="J98" s="3" t="n"/>
       <c r="K98" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Một policy tốt phải có quy tắc có thể kiểm thử và giữ trình tự cùng state cần thiết.</t>
+          <t>Các chính sách quản lý state hội thoại có kiểm soát gồm: Giữ N lượt gần nhất (sliding window) (a), Tóm tắt lượt cũ và giữ lượt gần đây (b), và Truy xuất state/fact liên quan theo ngữ cảnh (c). Xáo trộn hoặc xóa ngẫu nhiên làm hỏng tính mạch lạc.</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="H100" s="4" t="inlineStr">
         <is>
-          <t>3,4</t>
+          <t>1,2,5</t>
         </is>
       </c>
       <c r="I100" s="4" t="n">
@@ -5606,7 +5606,7 @@
       <c r="J100" s="3" t="n"/>
       <c r="K100" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Chỉ retry lỗi có khả năng tự thay đổi theo thời gian mà không cần sửa request hoặc credential.</t>
+          <t>Lỗi có thể retry là lỗi tạm thời có khả năng tự phục hồi: Timeout mạng tạm thời (a), Lỗi rate-limit 429 có Retry-After (b), và Lỗi 503 Service Unavailable tạm thời (e). Lỗi sai API key (c) và malformed schema (d) là lỗi 4xx cố định, không được retry.</t>
         </is>
       </c>
     </row>
@@ -5650,7 +5650,7 @@
       </c>
       <c r="H101" s="4" t="inlineStr">
         <is>
-          <t>1,4</t>
+          <t>1,2,3,4</t>
         </is>
       </c>
       <c r="I101" s="4" t="n">
@@ -5659,7 +5659,7 @@
       <c r="J101" s="3" t="n"/>
       <c r="K101" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Hỏi người kiểm thử cần biết gì để quyết định phần triển khai đạt hay không.</t>
+          <t>Đặc tả kiểm thử được cần: Định dạng/kích thước file và xử lý lỗi (a), Luồng giao diện/API (b), Ràng buộc bảo mật và lưu trữ (c), cùng Tiêu chí chấp nhận kiểm thử được (d).</t>
         </is>
       </c>
     </row>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="G102" s="3" t="n"/>
       <c r="H102" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I102" s="4" t="n">
         <v>60</v>
@@ -5705,7 +5705,7 @@
       <c r="J102" s="3" t="n"/>
       <c r="K102" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Một bài kiểm thử phải có thể trả kết quả đạt/không đạt từ hành vi cụ thể.</t>
+          <t>Tiêu chí chấp nhận kiểm thử được phải có đầu vào cụ thể, hành vi quan sát được và kết quả đạt/không đạt rõ ràng: 'Với CSV amount gồm 2, 3 và một dòng trống, hàm trả 5 và không gọi mạng'.</t>
         </is>
       </c>
     </row>
@@ -5749,7 +5749,7 @@
       </c>
       <c r="H103" s="4" t="inlineStr">
         <is>
-          <t>2,3</t>
+          <t>1,2,4</t>
         </is>
       </c>
       <c r="I103" s="4" t="n">
@@ -5758,7 +5758,7 @@
       <c r="J103" s="3" t="n"/>
       <c r="K103" s="3" t="inlineStr">
         <is>
-          <t>Phân tích theo nguyên lý thiết kế: Chọn hành động tạo bằng chứng quan sát được về hành vi so với contract.</t>
+          <t>Bằng chứng kiểm chứng trực tiếp gồm: Đối chiếu tiêu chí chấp nhận với code/test (a), Chạy bộ test đường bình thường và test biên/đối nghịch (b), và Kiểm tra hậu quả lỗi cùng regression test (d). Tin tưởng vì mã trông trôi chảy (c) hay hỏi lại mô hình (e) không tạo bằng chứng kiểm thử khách quan.</t>
         </is>
       </c>
     </row>

</xml_diff>